<commit_message>
Update Makefile and project structure for enhanced development workflow and testing. Added integration testing command, improved linting rules, and expanded help documentation. Refactored insights into decision insights, introduced validation thresholds, and updated schema for better clarity. Removed deprecated insights module and adjusted related tests. Updated case study benchmarks and validation logic for improved accuracy.
</commit_message>
<xml_diff>
--- a/docs/case_study/Interview Case Study - Finance Solution Developer - Model.xlsx
+++ b/docs/case_study/Interview Case Study - Finance Solution Developer - Model.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://seaspanltdca.sharepoint.com/sites/BusinessIntelligence/Shared Documents/Development/Finance Intelligence/99_Admin/Hiring/2026/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/joel/Github/Vessel/docs/case_study/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="579" documentId="8_{F221830E-9212-4E02-9CEA-7A222F6DB413}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B1518ACE-A882-4451-97DF-C42C06412649}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39287263-70DA-CF4A-AD31-2996F53EB3AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{81FA7CCF-C1FE-488E-8132-3F8F1B3B49A8}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="51200" windowHeight="28180" activeTab="2" xr2:uid="{81FA7CCF-C1FE-488E-8132-3F8F1B3B49A8}"/>
   </bookViews>
   <sheets>
     <sheet name="Input &amp; Output (Basic)" sheetId="1" r:id="rId1"/>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="68">
   <si>
     <t>Input Field</t>
   </si>
@@ -269,6 +269,9 @@
   </si>
   <si>
     <t>Inflation Rate Worst Case</t>
+  </si>
+  <si>
+    <t>test vessle #11</t>
   </si>
 </sst>
 </file>
@@ -276,14 +279,14 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="8">
-    <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0;[Red]\-&quot;$&quot;#,##0"/>
-    <numFmt numFmtId="44" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="165" formatCode="0&quot; years&quot;"/>
-    <numFmt numFmtId="166" formatCode="_-&quot;$&quot;* #,##0_-;\-&quot;$&quot;* #,##0_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="167" formatCode="_-&quot;$&quot;* #,##0_-;[Red]\-&quot;$&quot;* #,##0_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="168" formatCode="0.0&quot; years&quot;"/>
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0;[Red]\-&quot;$&quot;#,##0"/>
+    <numFmt numFmtId="165" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="166" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="167" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="168" formatCode="0&quot; years&quot;"/>
+    <numFmt numFmtId="169" formatCode="_-&quot;$&quot;* #,##0_-;\-&quot;$&quot;* #,##0_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="170" formatCode="_-&quot;$&quot;* #,##0_-;[Red]\-&quot;$&quot;* #,##0_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="171" formatCode="0.0&quot; years&quot;"/>
   </numFmts>
   <fonts count="15" x14ac:knownFonts="1">
     <font>
@@ -383,7 +386,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -393,6 +396,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF000000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -408,11 +417,11 @@
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -420,42 +429,44 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="9" fontId="6" fillId="0" borderId="0" xfId="3" applyFont="1"/>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="169" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" indent="2"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="169" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="169" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="170" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="170" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="169" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" indent="2"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="169" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="6" fontId="11" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="10" fontId="11" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="169" fontId="4" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="14" fontId="13" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="168" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="171" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="43" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="169" fontId="5" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="169" fontId="5" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -822,13 +833,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2A1069D-4443-4095-8164-81880652CE98}">
   <dimension ref="A1:B27"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="37.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="37.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -836,7 +847,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>12</v>
       </c>
@@ -844,7 +855,7 @@
         <v>46022</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
@@ -852,7 +863,7 @@
         <v>100000000</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
@@ -860,7 +871,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
@@ -868,7 +879,7 @@
         <v>5000000</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
@@ -876,7 +887,7 @@
         <v>50000</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
@@ -884,7 +895,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>44</v>
       </c>
@@ -892,7 +903,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
@@ -900,7 +911,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
@@ -908,7 +919,7 @@
         <v>5000000</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>17</v>
       </c>
@@ -916,7 +927,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>9</v>
       </c>
@@ -924,7 +935,7 @@
         <v>500000</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>14</v>
       </c>
@@ -932,7 +943,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>45</v>
       </c>
@@ -940,7 +951,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>33</v>
       </c>
@@ -948,7 +959,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" s="22" t="s">
         <v>34</v>
       </c>
@@ -957,7 +968,7 @@
         <v>4143625.443278688</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" s="22" t="s">
         <v>35</v>
       </c>
@@ -966,7 +977,7 @@
         <v>0.10585531076966781</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
         <v>63</v>
       </c>
@@ -974,7 +985,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>64</v>
       </c>
@@ -982,7 +993,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
         <v>65</v>
       </c>
@@ -990,7 +1001,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
         <v>66</v>
       </c>
@@ -1006,26 +1017,26 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{692B3806-0F68-4D15-90F5-807B9D5CD0CD}">
   <dimension ref="A1:AG31"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="31" style="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.140625" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.1640625" style="7" bestFit="1" customWidth="1"/>
     <col min="3" max="6" width="14" style="7" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.7109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.6640625" style="7" bestFit="1" customWidth="1"/>
     <col min="8" max="11" width="14" style="7" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.7109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.6640625" style="7" bestFit="1" customWidth="1"/>
     <col min="13" max="16" width="14" style="7" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="12.7109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12.6640625" style="7" bestFit="1" customWidth="1"/>
     <col min="18" max="21" width="14" style="7" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="12.7109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="12.6640625" style="7" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="14" style="7" bestFit="1" customWidth="1"/>
-    <col min="24" max="26" width="12.7109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="24" max="26" width="12.6640625" style="7" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="14" style="7" bestFit="1" customWidth="1"/>
-    <col min="28" max="33" width="11.7109375" style="7" bestFit="1" customWidth="1"/>
-    <col min="34" max="16384" width="8.7109375" style="7"/>
+    <col min="28" max="33" width="11.6640625" style="7" bestFit="1" customWidth="1"/>
+    <col min="34" max="16384" width="8.6640625" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" ht="15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.15">
       <c r="A1" s="26" t="s">
         <v>29</v>
       </c>
@@ -1062,7 +1073,7 @@
       <c r="AF1" s="27"/>
       <c r="AG1" s="27"/>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.15">
       <c r="A2" s="7" t="s">
         <v>16</v>
       </c>
@@ -1195,7 +1206,7 @@
         <v>57345</v>
       </c>
     </row>
-    <row r="3" spans="1:33" ht="15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:33" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="7" t="s">
         <v>18</v>
       </c>
@@ -1328,7 +1339,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.15">
       <c r="A4" s="7" t="s">
         <v>15</v>
       </c>
@@ -1525,7 +1536,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.15">
       <c r="A5" s="7" t="s">
         <v>13</v>
       </c>
@@ -1722,7 +1733,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:33" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:33" x14ac:dyDescent="0.15">
       <c r="A6" s="7" t="s">
         <v>40</v>
       </c>
@@ -1855,7 +1866,7 @@
         <v>2.5000803453253493</v>
       </c>
     </row>
-    <row r="7" spans="1:33" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:33" x14ac:dyDescent="0.15">
       <c r="A7" s="7" t="s">
         <v>41</v>
       </c>
@@ -1988,7 +1999,7 @@
         <v>19.194342495775089</v>
       </c>
     </row>
-    <row r="8" spans="1:33" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:33" x14ac:dyDescent="0.15">
       <c r="A8" s="7" t="s">
         <v>43</v>
       </c>
@@ -2121,7 +2132,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="9" spans="1:33" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:33" x14ac:dyDescent="0.15">
       <c r="A9" s="7" t="s">
         <v>42</v>
       </c>
@@ -2254,7 +2265,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="10" spans="1:33" s="11" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:33" s="11" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A10" s="11" t="s">
         <v>19</v>
       </c>
@@ -2387,7 +2398,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:33" s="21" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:33" s="21" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A11" s="20" t="s">
         <v>20</v>
       </c>
@@ -2520,7 +2531,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:33" s="11" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:33" s="11" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A12" s="11" t="s">
         <v>38</v>
       </c>
@@ -2653,7 +2664,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:33" s="21" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:33" s="21" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A13" s="20" t="s">
         <v>21</v>
       </c>
@@ -2786,7 +2797,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:33" s="11" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:33" s="11" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A14" s="11" t="s">
         <v>23</v>
       </c>
@@ -2919,7 +2930,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:33" s="21" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:33" s="21" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A15" s="20" t="s">
         <v>22</v>
       </c>
@@ -3052,7 +3063,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:33" s="11" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:33" s="11" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A16" s="11" t="s">
         <v>24</v>
       </c>
@@ -3185,8 +3196,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:33" s="11" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="18" spans="1:33" ht="15" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:33" s="11" customFormat="1" x14ac:dyDescent="0.15"/>
+    <row r="18" spans="1:33" x14ac:dyDescent="0.15">
       <c r="A18" s="26" t="s">
         <v>28</v>
       </c>
@@ -3223,7 +3234,7 @@
       <c r="AF18" s="28"/>
       <c r="AG18" s="28"/>
     </row>
-    <row r="19" spans="1:33" s="15" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:33" s="15" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A19" s="15" t="s">
         <v>26</v>
       </c>
@@ -3356,7 +3367,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:33" s="15" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:33" s="15" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A20" s="15" t="s">
         <v>27</v>
       </c>
@@ -3489,7 +3500,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:33" s="14" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:33" s="14" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A21" s="12" t="s">
         <v>11</v>
       </c>
@@ -3622,7 +3633,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:33" s="14" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:33" s="14" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A22" s="12" t="s">
         <v>10</v>
       </c>
@@ -3755,7 +3766,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:33" s="15" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:33" s="15" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A23" s="15" t="s">
         <v>25</v>
       </c>
@@ -3888,7 +3899,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:33" s="15" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:33" s="15" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A24" s="15" t="s">
         <v>37</v>
       </c>
@@ -4021,7 +4032,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:33" ht="15" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:33" x14ac:dyDescent="0.15">
       <c r="A26" s="26" t="s">
         <v>30</v>
       </c>
@@ -4058,7 +4069,7 @@
       <c r="AF26" s="27"/>
       <c r="AG26" s="27"/>
     </row>
-    <row r="27" spans="1:33" s="14" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:33" s="14" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A27" s="12" t="s">
         <v>31</v>
       </c>
@@ -4191,7 +4202,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:33" s="14" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:33" s="14" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A28" s="12" t="s">
         <v>32</v>
       </c>
@@ -4324,7 +4335,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:33" s="15" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:33" s="15" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A29" s="15" t="s">
         <v>36</v>
       </c>
@@ -4457,7 +4468,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:33" s="15" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:33" s="15" customFormat="1" x14ac:dyDescent="0.15">
       <c r="A31" s="15" t="s">
         <v>39</v>
       </c>
@@ -4607,30 +4618,30 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06BB2ACA-81BF-4CC8-9D8F-0AB13D47078D}">
-  <dimension ref="A1:R11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:R12"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="22.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="25.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.5" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="20" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="38.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="38.6640625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="24" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="25.5703125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="28.140625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="29.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="25.5" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="28.1640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="29.5" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="22.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -4686,7 +4697,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>46</v>
       </c>
@@ -4743,7 +4754,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>47</v>
       </c>
@@ -4801,7 +4812,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>48</v>
       </c>
@@ -4812,7 +4823,7 @@
         <v>12500</v>
       </c>
       <c r="D4" s="6">
-        <f t="shared" ref="D4:D11" si="1">EOMONTH(D3,3)</f>
+        <f t="shared" ref="D4:D12" si="1">EOMONTH(D3,3)</f>
         <v>44834</v>
       </c>
       <c r="E4" s="25">
@@ -4859,7 +4870,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="5" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>49</v>
       </c>
@@ -4916,7 +4927,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="6" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>50</v>
       </c>
@@ -4973,7 +4984,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="7" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>51</v>
       </c>
@@ -5030,7 +5041,7 @@
         <v>1.05</v>
       </c>
     </row>
-    <row r="8" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>52</v>
       </c>
@@ -5087,14 +5098,14 @@
         <v>1.05</v>
       </c>
     </row>
-    <row r="9" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>53</v>
       </c>
       <c r="B9" s="30">
         <v>8000</v>
       </c>
-      <c r="C9" s="30" t="s">
+      <c r="C9" s="34" t="s">
         <v>58</v>
       </c>
       <c r="D9" s="6">
@@ -5106,7 +5117,7 @@
       <c r="F9" s="4">
         <v>25</v>
       </c>
-      <c r="G9" s="31" t="e">
+      <c r="G9" s="33" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
@@ -5144,7 +5155,7 @@
         <v>0.78</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>54</v>
       </c>
@@ -5202,7 +5213,7 @@
         <v>0.78</v>
       </c>
     </row>
-    <row r="11" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>55</v>
       </c>
@@ -5257,6 +5268,64 @@
         <v>61</v>
       </c>
       <c r="R11" s="32">
+        <v>0.78</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B12" s="30">
+        <v>8000</v>
+      </c>
+      <c r="C12" s="30">
+        <v>13095</v>
+      </c>
+      <c r="D12" s="6">
+        <f t="shared" si="1"/>
+        <v>46022</v>
+      </c>
+      <c r="E12" s="25">
+        <v>9000000</v>
+      </c>
+      <c r="F12" s="4">
+        <v>25</v>
+      </c>
+      <c r="G12" s="31">
+        <f t="shared" ref="G12" si="2">C12*400</f>
+        <v>5238000</v>
+      </c>
+      <c r="H12" s="25">
+        <v>45500</v>
+      </c>
+      <c r="I12" s="3">
+        <v>365</v>
+      </c>
+      <c r="J12" s="5">
+        <v>0.02</v>
+      </c>
+      <c r="K12" s="25">
+        <v>10500</v>
+      </c>
+      <c r="L12" s="25">
+        <v>5240000</v>
+      </c>
+      <c r="M12" s="4">
+        <v>5</v>
+      </c>
+      <c r="N12" s="25">
+        <v>500000</v>
+      </c>
+      <c r="O12" s="5">
+        <v>0.03</v>
+      </c>
+      <c r="P12" s="5">
+        <v>0.1</v>
+      </c>
+      <c r="Q12" s="31" t="s">
+        <v>61</v>
+      </c>
+      <c r="R12" s="32">
         <v>0.78</v>
       </c>
     </row>
@@ -5267,6 +5336,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ec1e0b3d-e6d4-4d60-8336-06175c753c05">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="cb33da3d-792e-415a-9ec2-59bdff1453f2" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -5275,7 +5355,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B1185F8B81323C419B9D13BECBC00B5F" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="0370c41719017e07fc235c27441ca214">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="ec1e0b3d-e6d4-4d60-8336-06175c753c05" xmlns:ns3="cb33da3d-792e-415a-9ec2-59bdff1453f2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="eae17a4802d55bc3bdcf418c9e0e10f0" ns2:_="" ns3:_="">
     <xsd:import namespace="ec1e0b3d-e6d4-4d60-8336-06175c753c05"/>
@@ -5516,18 +5596,18 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ec1e0b3d-e6d4-4d60-8336-06175c753c05">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="cb33da3d-792e-415a-9ec2-59bdff1453f2" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{390D22E3-FCDF-4307-9243-D875F504B570}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="ec1e0b3d-e6d4-4d60-8336-06175c753c05"/>
+    <ds:schemaRef ds:uri="cb33da3d-792e-415a-9ec2-59bdff1453f2"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D8181EDB-E5E3-43EF-B217-EB703F8D4C16}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -5535,7 +5615,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{32C13A5E-FDF6-49B2-A8D5-4F61FB0014DE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5552,15 +5632,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{390D22E3-FCDF-4307-9243-D875F504B570}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="ec1e0b3d-e6d4-4d60-8336-06175c753c05"/>
-    <ds:schemaRef ds:uri="cb33da3d-792e-415a-9ec2-59bdff1453f2"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>